<commit_message>
docs: atualiza readme e estrutura de modelagem relacional
- Atualização do README para refletir o progresso da visualização de dados.

Implementação de relacionamentos 1:N no Power BI (Vendas x Produtos x Vendedores).

Normalização de dados via IDs para garantir integridade referencial.
</commit_message>
<xml_diff>
--- a/SQL/PostgreSQL/Projeto Vendas/Dados/base_vendas.xlsx
+++ b/SQL/PostgreSQL/Projeto Vendas/Dados/base_vendas.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
   <si>
     <t>id_venda</t>
   </si>
@@ -141,7 +141,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -640,7 +640,7 @@
     </xf>
     <xf numFmtId="2" fontId="17" fillId="29" borderId="0" xfId="38" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="17" fillId="29" borderId="0" xfId="38" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="17" fillId="29" borderId="0" xfId="38" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="29" borderId="0" xfId="38" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="17" fillId="29" borderId="0" xfId="38" applyNumberFormat="1" applyAlignment="1">
@@ -693,22 +693,6 @@
   </cellStyles>
   <dxfs count="18">
     <dxf>
-      <numFmt numFmtId="169" formatCode="&quot;R$&quot;\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="&quot;R$&quot;\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center"/>
     </dxf>
@@ -731,6 +715,14 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -749,6 +741,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -767,6 +760,13 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -996,19 +996,19 @@
     <tableColumn id="1" name="id_venda" dataDxfId="14" totalsRowDxfId="13" dataCellStyle="Ênfase6"/>
     <tableColumn id="2" name="id_cliente" dataDxfId="12" totalsRowDxfId="11" dataCellStyle="Ênfase6"/>
     <tableColumn id="3" name="id_vendedor" dataDxfId="10" totalsRowDxfId="9" dataCellStyle="Ênfase6"/>
-    <tableColumn id="6" name="id_produto" dataDxfId="7" dataCellStyle="Ênfase6"/>
-    <tableColumn id="4" name="nome_produto" totalsRowFunction="custom" dataDxfId="2" totalsRowDxfId="8" dataCellStyle="Ênfase6">
+    <tableColumn id="6" name="id_produto" dataDxfId="8" dataCellStyle="Ênfase6"/>
+    <tableColumn id="4" name="nome_produto" totalsRowFunction="custom" dataDxfId="7" totalsRowDxfId="6" dataCellStyle="Ênfase6">
       <calculatedColumnFormula>VLOOKUP(Tabela1[[#This Row],[id_produto]],'[1]Preparando Tabela de Produtos p'!$A$1:$C$11,2,0)</calculatedColumnFormula>
       <totalsRowFormula>SUBTOTAL(109,E2:E31)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" name="preco_unitario" dataDxfId="0" totalsRowDxfId="5" dataCellStyle="Ênfase6">
+    <tableColumn id="9" name="preco_unitario" dataDxfId="5" totalsRowDxfId="4" dataCellStyle="Ênfase6">
       <calculatedColumnFormula>VLOOKUP(Tabela1[[#This Row],[id_produto]],'[1]Preparando Tabela de Produtos p'!$A$1:$C$11,3,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" name="quantidade" dataDxfId="1" dataCellStyle="Ênfase6"/>
-    <tableColumn id="8" name="valor" dataDxfId="3" totalsRowDxfId="6" dataCellStyle="Ênfase6">
+    <tableColumn id="10" name="quantidade" dataDxfId="3" dataCellStyle="Ênfase6"/>
+    <tableColumn id="8" name="valor" dataDxfId="2" totalsRowDxfId="1" dataCellStyle="Ênfase6">
       <calculatedColumnFormula>Tabela1[[#This Row],[quantidade]]*Tabela1[[#This Row],[preco_unitario]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" name="data_venda" dataDxfId="4" dataCellStyle="Ênfase6"/>
+    <tableColumn id="5" name="data_venda" dataDxfId="0" dataCellStyle="Ênfase6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1457,7 +1457,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C5" s="1">
         <v>5</v>
@@ -1490,7 +1490,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C6" s="1">
         <v>6</v>
@@ -1514,7 +1514,7 @@
         <v>2300</v>
       </c>
       <c r="I6" s="5">
-        <v>46262</v>
+        <v>46198</v>
       </c>
       <c r="M6" s="8"/>
     </row>
@@ -1523,7 +1523,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C7" s="1">
         <v>7</v>
@@ -1556,7 +1556,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C8" s="1">
         <v>2</v>
@@ -1590,7 +1590,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="1">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C9" s="1">
         <v>3</v>
@@ -1722,7 +1722,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C13" s="1">
         <v>7</v>
@@ -1754,8 +1754,8 @@
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>8</v>
+      <c r="B14" s="1">
+        <v>6</v>
       </c>
       <c r="C14" s="1">
         <v>2</v>
@@ -1787,8 +1787,8 @@
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>6</v>
+      <c r="B15" s="1">
+        <v>7</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>8</v>
@@ -1812,7 +1812,7 @@
         <v>2900</v>
       </c>
       <c r="I15" s="5">
-        <v>46265</v>
+        <v>46193</v>
       </c>
       <c r="M15" s="8"/>
     </row>
@@ -1820,8 +1820,8 @@
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>11</v>
+      <c r="B16" s="1">
+        <v>8</v>
       </c>
       <c r="C16" s="1">
         <v>4</v>
@@ -1854,7 +1854,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="1">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C17" s="1">
         <v>5</v>
@@ -1970,11 +1970,11 @@
         <v>1100</v>
       </c>
       <c r="G20" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H20" s="9">
         <f>Tabela1[[#This Row],[quantidade]]*Tabela1[[#This Row],[preco_unitario]]</f>
-        <v>1100</v>
+        <v>3300</v>
       </c>
       <c r="I20" s="5">
         <v>46228</v>
@@ -1986,7 +1986,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>8</v>
@@ -2018,8 +2018,8 @@
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>8</v>
+      <c r="B22" s="1">
+        <v>6</v>
       </c>
       <c r="C22" s="1">
         <v>4</v>
@@ -2051,8 +2051,8 @@
       <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>6</v>
+      <c r="B23" s="1">
+        <v>7</v>
       </c>
       <c r="C23" s="1">
         <v>5</v>
@@ -2069,11 +2069,11 @@
         <v>1150</v>
       </c>
       <c r="G23" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H23" s="9">
         <f>Tabela1[[#This Row],[quantidade]]*Tabela1[[#This Row],[preco_unitario]]</f>
-        <v>1150</v>
+        <v>2300</v>
       </c>
       <c r="I23" s="5">
         <v>46218</v>
@@ -2084,8 +2084,8 @@
       <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>11</v>
+      <c r="B24" s="1">
+        <v>8</v>
       </c>
       <c r="C24" s="1">
         <v>6</v>
@@ -2118,7 +2118,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="1">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C25" s="1">
         <v>7</v>

</xml_diff>